<commit_message>
Modification des fonctions de calcul de seuil
</commit_message>
<xml_diff>
--- a/docs/Balance UM  2023 VF(N-1).xlsx
+++ b/docs/Balance UM  2023 VF(N-1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mariam Latifa DALLA\Documents\cac-perform\cac-perform-main\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mariam Latifa DALLA\Desktop\Cac_perform-main\Cac_perform-main\cac-perform-main\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38F617BB-4226-42D3-84EB-A3A259677125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1AC8126-1946-47BF-94CE-6A1217529924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{55DA9684-6164-404E-8838-BEDA660D5D98}"/>
   </bookViews>
@@ -2595,15 +2595,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100030E4331D3E9AB4EB662C8267643069E" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="6bbc25e2cde7fb85d35286a54bbd7e10">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="b2b586be-b205-4674-b1e5-6a2eaa363eda" xmlns:ns4="40d7a5e3-7718-4dc5-852f-d459693408a7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1a373a4da292abf1c0fe79ab7cbd0238" ns3:_="" ns4:_="">
     <xsd:import namespace="b2b586be-b205-4674-b1e5-6a2eaa363eda"/>
@@ -2824,6 +2815,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2833,14 +2833,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBACF1FD-985C-44D6-AAEE-64E55C661624}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F066AFF2-94CE-4F7F-9341-D82D91CDC2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2859,6 +2851,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBACF1FD-985C-44D6-AAEE-64E55C661624}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E22F1C8-6585-41E7-9783-A1FEABD8828F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Revert "Modification des fonctions de calcul de seuil"
This reverts commit 5110468132f941234f924bef8071ca3ecba79e7f.
</commit_message>
<xml_diff>
--- a/docs/Balance UM  2023 VF(N-1).xlsx
+++ b/docs/Balance UM  2023 VF(N-1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mariam Latifa DALLA\Desktop\Cac_perform-main\Cac_perform-main\cac-perform-main\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mariam Latifa DALLA\Documents\cac-perform\cac-perform-main\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1AC8126-1946-47BF-94CE-6A1217529924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{38F617BB-4226-42D3-84EB-A3A259677125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{55DA9684-6164-404E-8838-BEDA660D5D98}"/>
   </bookViews>
@@ -2595,6 +2595,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100030E4331D3E9AB4EB662C8267643069E" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="6bbc25e2cde7fb85d35286a54bbd7e10">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="b2b586be-b205-4674-b1e5-6a2eaa363eda" xmlns:ns4="40d7a5e3-7718-4dc5-852f-d459693408a7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1a373a4da292abf1c0fe79ab7cbd0238" ns3:_="" ns4:_="">
     <xsd:import namespace="b2b586be-b205-4674-b1e5-6a2eaa363eda"/>
@@ -2815,15 +2824,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2833,6 +2833,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBACF1FD-985C-44D6-AAEE-64E55C661624}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F066AFF2-94CE-4F7F-9341-D82D91CDC2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2851,14 +2859,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBACF1FD-985C-44D6-AAEE-64E55C661624}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E22F1C8-6585-41E7-9783-A1FEABD8828F}">
   <ds:schemaRefs>

</xml_diff>